<commit_message>
Corrida | ARG-IL5 | 2026-06-17 09:53:54.109853
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IL5_out.xlsx
+++ b/indicadores/ARG-IL5_out.xlsx
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice de capacidad instalada general de la industria argentina</t>
+    <t xml:space="preserve">Índice de capacidad instalada general de la industria</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -119,7 +119,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -27157,4 +27157,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1747652-30A6-4B76-8207-9D35BEA9511B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{754B6BDC-4B94-4737-9914-BAB03BF6B903}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8262495C-7826-42A3-91E9-7ADC99AFC577}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-IL5 | 2026-06-17 09:58:52.330838
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IL5_out.xlsx
+++ b/indicadores/ARG-IL5_out.xlsx
@@ -119,7 +119,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -27157,237 +27157,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1747652-30A6-4B76-8207-9D35BEA9511B}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{754B6BDC-4B94-4737-9914-BAB03BF6B903}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8262495C-7826-42A3-91E9-7ADC99AFC577}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-IL5 | 2026-06-17 11:05:19.565484
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IL5_out.xlsx
+++ b/indicadores/ARG-IL5_out.xlsx
@@ -27157,4 +27157,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F9C9F0D-C83E-4296-9B28-57B2EAC9E864}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{856F6A35-9E7C-4E66-9D33-82601EA66841}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2200234E-AD09-44FE-8622-C74A97DB441C}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-IL5 | 2026-06-17 11:12:43.15711
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IL5_out.xlsx
+++ b/indicadores/ARG-IL5_out.xlsx
@@ -27157,237 +27157,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F9C9F0D-C83E-4296-9B28-57B2EAC9E864}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{856F6A35-9E7C-4E66-9D33-82601EA66841}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2200234E-AD09-44FE-8622-C74A97DB441C}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-IL5 | 2026-06-18 09:52:34.634
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IL5_out.xlsx
+++ b/indicadores/ARG-IL5_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/06/2026</t>
+    <t xml:space="preserve">18/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2146,9 +2146,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -2160,14 +2158,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
+      <c r="A9"/>
       <c r="B9"/>
       <c r="C9"/>
-      <c r="D9" t="n">
-        <v>0.510061557114689</v>
-      </c>
+      <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9"/>
@@ -2177,13 +2171,11 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
@@ -2192,10 +2184,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" t="n">
+        <v>0.519143609599933</v>
+      </c>
       <c r="E11"/>
       <c r="F11"/>
       <c r="G11"/>
@@ -2205,11 +2201,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
@@ -2218,14 +2216,10 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
+      <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" t="n">
-        <v>0.260162792046261</v>
-      </c>
+      <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
@@ -2234,7 +2228,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14">
-      <c r="A14"/>
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -2247,11 +2243,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" t="n">
+        <v>0.269510087388447</v>
+      </c>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
@@ -2260,9 +2258,7 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
+      <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -2275,7 +2271,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2289,13 +2285,11 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
-      <c r="D18" t="n">
-        <v>0.0680930471015797</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18"/>
       <c r="G18"/>
@@ -2305,7 +2299,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2324,7 +2318,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000385280915004682</v>
+        <v>0.0383996083607185</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2334,7 +2328,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
@@ -2346,10 +2342,14 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22">
-      <c r="A22"/>
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
       <c r="B22"/>
       <c r="C22"/>
-      <c r="D22"/>
+      <c r="D22" t="n">
+        <v>0.000145560286402963</v>
+      </c>
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22"/>
@@ -26985,7 +26985,7 @@
         <v>519</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0390504071211762</v>
+        <v>0.0301293831384062</v>
       </c>
     </row>
     <row r="6">
@@ -26993,7 +26993,7 @@
         <v>520</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0733211986975836</v>
+        <v>0.0621057309743825</v>
       </c>
     </row>
     <row r="7">
@@ -27001,7 +27001,7 @@
         <v>521</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.11802881538133</v>
+        <v>0.107215191876675</v>
       </c>
     </row>
     <row r="8">
@@ -27009,7 +27009,7 @@
         <v>522</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.18153219483201</v>
+        <v>0.17028666603047</v>
       </c>
     </row>
     <row r="9">
@@ -27017,7 +27017,7 @@
         <v>523</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.24084157241065</v>
+        <v>0.231137689034371</v>
       </c>
     </row>
     <row r="10">
@@ -27025,7 +27025,7 @@
         <v>524</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.301341074979746</v>
+        <v>0.299423252182022</v>
       </c>
     </row>
     <row r="11">
@@ -27033,7 +27033,7 @@
         <v>525</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.388846819474096</v>
+        <v>0.390678872248798</v>
       </c>
     </row>
     <row r="12">
@@ -27041,7 +27041,7 @@
         <v>526</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.447533673658024</v>
+        <v>0.446174861042707</v>
       </c>
     </row>
     <row r="13">
@@ -27049,7 +27049,7 @@
         <v>527</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.474233909404269</v>
+        <v>0.47690694712617</v>
       </c>
     </row>
     <row r="14">
@@ -27057,7 +27057,7 @@
         <v>528</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.510061557114689</v>
+        <v>0.519143609599933</v>
       </c>
     </row>
     <row r="15">
@@ -27065,7 +27065,7 @@
         <v>529</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.463050301191295</v>
+        <v>0.469715494161817</v>
       </c>
     </row>
     <row r="16">
@@ -27073,7 +27073,7 @@
         <v>530</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.353211043012577</v>
+        <v>0.356902543917561</v>
       </c>
     </row>
     <row r="17">
@@ -27081,7 +27081,7 @@
         <v>531</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.256987263478015</v>
+        <v>0.26003662428982</v>
       </c>
     </row>
     <row r="18">
@@ -27089,7 +27089,7 @@
         <v>532</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.145183754671099</v>
+        <v>0.14668597764962</v>
       </c>
     </row>
     <row r="19">
@@ -27097,7 +27097,7 @@
         <v>533</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.034981898007187</v>
+        <v>0.0368242265538172</v>
       </c>
     </row>
     <row r="20">
@@ -27105,7 +27105,7 @@
         <v>534</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0410792174140544</v>
+        <v>-0.0388925654958154</v>
       </c>
     </row>
     <row r="21">
@@ -27113,7 +27113,7 @@
         <v>535</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0986341699909351</v>
+        <v>-0.0997456169264908</v>
       </c>
     </row>
     <row r="22">
@@ -27121,7 +27121,7 @@
         <v>536</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.140140904438804</v>
+        <v>-0.141381696727311</v>
       </c>
     </row>
     <row r="23">
@@ -27129,7 +27129,7 @@
         <v>537</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.15831641180546</v>
+        <v>-0.157221931168126</v>
       </c>
     </row>
     <row r="24">
@@ -27157,4 +27157,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B74837-FC5A-4DC5-BDAE-2911FCC9BED4}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9613653C-0043-4572-A82C-A31385D2D876}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CBBBC18-1C94-46A0-8802-294419A27B3F}"/>
 </file>
</xml_diff>